<commit_message>
Migrate from SQLite to PostgreSQL - eliminate database locking
</commit_message>
<xml_diff>
--- a/Bugs.xlsx
+++ b/Bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbklitgaard/job_hunter_web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005B8889-4D82-4A4B-976A-235809EFCF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5411663-F587-2B44-80D9-97DA203DD21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35020" yWindow="-5400" windowWidth="29400" windowHeight="17440" xr2:uid="{6ACB163A-A46A-7F49-B2A0-BA3E5AC50E99}"/>
   </bookViews>
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -343,128 +343,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -507,11 +390,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -526,12 +409,36 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1030,7 +937,7 @@
         <v>12</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>24</v>
@@ -1212,7 +1119,7 @@
       <c r="D17" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="7" t="s">
         <v>31</v>
       </c>
       <c r="F17" s="6" t="s">
@@ -1571,7 +1478,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>67</v>
@@ -1651,7 +1558,7 @@
         <v>11</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>70</v>
@@ -1846,42 +1753,42 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G31" xr:uid="{2E964C1B-192B-AF4A-81A6-4BFC861E48E5}"/>
-  <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="containsText" dxfId="16" priority="10" operator="containsText" text="Open">
-      <formula>NOT(ISERROR(SEARCH("Open",D1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="9" operator="containsText" text="New">
-      <formula>NOT(ISERROR(SEARCH("New",D1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="8" operator="containsText" text="Fixed">
-      <formula>NOT(ISERROR(SEARCH("Fixed",D1)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="containsText" dxfId="10" priority="7" operator="containsText" text="1">
-      <formula>NOT(ISERROR(SEARCH("1",B1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="6" operator="containsText" text="2">
-      <formula>NOT(ISERROR(SEARCH("2",B1)))</formula>
-    </cfRule>
     <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="3">
       <formula>NOT(ISERROR(SEARCH("3",B1)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24">
-    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="Critical">
-      <formula>NOT(ISERROR(SEARCH("Critical",E24)))</formula>
+    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="2">
+      <formula>NOT(ISERROR(SEARCH("2",B1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="1">
+      <formula>NOT(ISERROR(SEARCH("1",B1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Critical">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Medium">
+      <formula>NOT(ISERROR(SEARCH("Medium",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="High">
+      <formula>NOT(ISERROR(SEARCH("High",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Critical">
       <formula>NOT(ISERROR(SEARCH("Critical",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="High">
-      <formula>NOT(ISERROR(SEARCH("High",C1)))</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="containsText" dxfId="3" priority="8" operator="containsText" text="Fixed">
+      <formula>NOT(ISERROR(SEARCH("Fixed",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Medium">
-      <formula>NOT(ISERROR(SEARCH("Medium",C1)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="9" operator="containsText" text="New">
+      <formula>NOT(ISERROR(SEARCH("New",D1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="10" operator="containsText" text="Open">
+      <formula>NOT(ISERROR(SEARCH("Open",D1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24">
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Critical">
+      <formula>NOT(ISERROR(SEARCH("Critical",E24)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>